<commit_message>
Job Scraper v5: 3 co | 30 jobs | 05-15 16:50
</commit_message>
<xml_diff>
--- a/download/Bewerbungen_Junior_IT.xlsx
+++ b/download/Bewerbungen_Junior_IT.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Statistiken" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bewerbungen'!$A$1:$N$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bewerbungen'!$A$1:$N$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:N31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1807,9 +1807,736 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>ercas Software Solutions GmbH</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Bilanzbuchhalter (m/w/d) Vollzeit in</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Bilanzbuchhalter (m/w/d) Vollzeit in
+                    Nürnberg Kategorie: Kaufmännisch</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>kontakt@ercas.com</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr"/>
+      <c r="G21" s="2" t="inlineStr"/>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>https://ercas.com/</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Nürnberger Str. 71, 91052 Erlangen, Deutschland, 91052 Erlangen</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Bilanzbuchhalter (m/w/d) Vollzeit in in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>https://ercas.com/job-bilanzbuchhalter-m-w-d-nuernberg-3678</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15 16:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>ercas Software Solutions GmbH</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Architekt*in Wohnungsbau (m/w/d) Vollzeit in</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Architekt*in Wohnungsbau (m/w/d) Vollzeit in
+                    Nürnberg Kategorie: Technisch</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>kontakt@ercas.com</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr"/>
+      <c r="G22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>https://ercas.com/</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Nürnberger Str. 71, 91052 Erlangen, Deutschland, 91052 Erlangen</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Architekt*in Wohnungsbau (m/w/d) Vollzeit in in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>https://ercas.com/job-architekt-in-wohnungsbau-m-w-d-nuernberg-3676</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15 16:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>ercas Software Solutions GmbH</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Baukalkulator (m/w/d) Vollzeit in</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Baukalkulator (m/w/d) Vollzeit in
+                    Nürnberg Kategorie: Technisch</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>kontakt@ercas.com</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="inlineStr"/>
+      <c r="G23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>https://ercas.com/</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Nürnberger Str. 71, 91052 Erlangen, Deutschland, 91052 Erlangen</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Baukalkulator (m/w/d) Vollzeit in in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>https://ercas.com/job-baukalkulator-m-w-d-nuernberg-3675</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15 16:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>ercas Software Solutions GmbH</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Wirtschaftsingenieur (m/w/d) – Unit A / B / C Vollzeit in</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Wirtschaftsingenieur (m/w/d) – Unit A / B / C Vollzeit in
+                    Nürnberg Kategorie: Kaufmännisch</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>kontakt@ercas.com</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr"/>
+      <c r="G24" s="2" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>https://ercas.com/</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Nürnberger Str. 71, 91052 Erlangen, Deutschland, 91052 Erlangen</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Wirtschaftsingenieur (m/w/d) – Unit A / B / C Vollzeit in in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>https://ercas.com/job-wirtschaftsingenieur-m-w-d-unit-a-b-c-nuernberg-3673</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15 16:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>ercas Software Solutions GmbH</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Wirtschaftsingenieur (m/w/d) – Unit A / B / C</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Wirtschaftsingenieur (m/w/d) – Unit A / B / C</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>kontakt@ercas.com</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr"/>
+      <c r="F25" s="2" t="inlineStr"/>
+      <c r="G25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>https://ercas.com/</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Nürnberger Str. 71, 91052 Erlangen, Deutschland, 91052 Erlangen</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Wirtschaftsingenieur (m/w/d) – Unit A / B / C in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>https://ercas.com/job-wirtschaftsingenieur-m-w-d-unit-a-b-c-nuernberg-3673</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15 16:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Schaeffler Technologies AG &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Duales Studium (DHBW) - Data Science und künstliche Intelligenz (m/w/d) 2026</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Quelle: Arbeitsagentur</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>info.de@schaeffler.com</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr"/>
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>http://www.schaeffler.de/</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Buckenhof</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Duales Studium (DHBW) - Data Science und künstliche Intelligenz (m/w/d) 2026 in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15 16:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>M.IT Connect GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Ausbildung zum Kaufmann für IT-System-Management (m/w/d)</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Ausbildung zum Kaufmann für IT-System-Management (m/w/d)            
+              Du interessierst dich für IT, aber auch für Beratung, Verkauf und Projektmanagement? Wir sind uns sicher, eine Ausbildung zum Kaufmann (m/w/d) für IT-System-Management wird dir dann richtig viel Freude machen!
+           Mehr erfahren</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr"/>
+      <c r="E27" s="2" t="inlineStr"/>
+      <c r="F27" s="2" t="inlineStr"/>
+      <c r="G27" s="2" t="inlineStr"/>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>http://www.m-it-connect.de/</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>Forchheim</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Ausbildung zum Kaufmann für IT-System-Management (m/w/d) in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.m-it-connect.de/stellenangebot.php?id=8a7ec3ad94e870850194f591f4bf0436</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15 16:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>M.IT Connect GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>IT-Consultant (m/w/d) für Microsoft 365</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>IT-Consultant (m/w/d) für Microsoft 365            
+              Du kennst dich mit Microsoft 365 bestens aus? Du liebst technologische Herausforderungen? Und hast Lust, diese in spannenden und anspruchsvollen Kundenprojekten umzusetzen? Das sind großartige Voraussetzungen, um bei uns als IT-Consultant deine Karriere zu starten.
+           Mehr erfahren</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr"/>
+      <c r="G28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>http://www.m-it-connect.de/</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>Forchheim</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als IT-Consultant (m/w/d) für Microsoft 365 in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.m-it-connect.de/stellenangebot.php?id=8a7ec14f8e273aea018e8475f03e1298</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15 16:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>M.IT Connect GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Ausbildung zum Fachinformatiker (m/w/d) für Systemintegration</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Ausbildung zum Fachinformatiker (m/w/d) für Systemintegration            
+              Es reizt dich, zu erfahren, wie IT-Systeme hinter den Kulissen funktionieren? Du hast Lust darauf, moderne Netzwerke einzurichten, Server aufzusetzen und dafür zu sorgen, dass Hard- und Software perfekt zusammenspielen? Als Fachinformatiker (m/w/d) für Systemintegration wirst du bei uns zum Experten für IT-Infrastrukturen  ...
+           Mehr erfahren</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr"/>
+      <c r="E29" s="2" t="inlineStr"/>
+      <c r="F29" s="2" t="inlineStr"/>
+      <c r="G29" s="2" t="inlineStr"/>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>http://www.m-it-connect.de/</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>Forchheim</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Ausbildung zum Fachinformatiker (m/w/d) für Systemintegration in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.m-it-connect.de/stellenangebot.php?id=8a7ec3ad94e870850194f57e8acd0373</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15 16:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>M.IT Connect GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Ausbildung zum Fachinformatiker (m/w/d) für Daten- und Prozessanalyse</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Ausbildung zum Fachinformatiker (m/w/d) für Daten- und Prozessanalyse            
+              Du willst verstehen, wie man Prozesse mit (den richtigen) Daten optimieren kann - und lernen, wie moderne Unternehmen IT gezielt einsetzen? Von der Analyse bis zur Lösung? Dann starte deine Ausbildung zum Fachinformatiker (m/w/d) für Daten- und Prozessanalyse bei M.IT Connect! 
+           Mehr erfahren</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr"/>
+      <c r="G30" s="2" t="inlineStr"/>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>http://www.m-it-connect.de/</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>Forchheim</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Ausbildung zum Fachinformatiker (m/w/d) für Daten- und Prozessanalyse in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.m-it-connect.de/stellenangebot.php?id=8a7ec05797b40d8c0197e4fa531b0f4a</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15 16:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>M.IT Connect GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Ausbildung zum Fachinformatiker (m/w/d) für Anwendungsentwicklung</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Ausbildung zum Fachinformatiker (m/w/d) für Anwendungsentwicklung            
+              Du willst Programme und Apps nicht nur nutzen, sondern sie selbst entwickeln? Absolviere einfach unsere Ausbildung zum Fachinformatiker bzw. zur Fachinformatikerin für Anwendungsentwicklung und erfahre, wie aus Code smarte Softwarelösungen werden – von der ersten Idee über die Programmierung bis zum Go-Live. Egal, ob  ...
+           Mehr erfahren</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr"/>
+      <c r="E31" s="2" t="inlineStr"/>
+      <c r="F31" s="2" t="inlineStr"/>
+      <c r="G31" s="2" t="inlineStr"/>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>http://www.m-it-connect.de/</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>Forchheim</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Ausbildung zum Fachinformatiker (m/w/d) für Anwendungsentwicklung in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.m-it-connect.de/stellenangebot.php?id=8a7ec3ad94e870850194f3f02324020e</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15 16:50</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N20"/>
-  <conditionalFormatting sqref="H2:H20">
+  <autoFilter ref="A1:N31"/>
+  <conditionalFormatting sqref="H2:H31">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Zusage"</formula>
     </cfRule>
@@ -1826,13 +2553,13 @@
       <formula>"Interview absolviert"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M2:M20">
+  <conditionalFormatting sqref="M2:M31">
     <cfRule type="cellIs" priority="6" operator="equal" dxfId="0">
       <formula>"Ja"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2 H3 H4 H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2 H3 H4 H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Offen,Beworben,Interview eingeplant,Interview absolviert,Zusage,Absage,Kontaktiert,Wiedervorlage,Kein Interesse"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1846,7 +2573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2480,6 +3207,360 @@
         <is>
           <t>Sehr geehrter Damen und Herren,
 ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Ingenieur für Automatisierungstechnik (m/w/d) | Angebotsnummer: 11751 in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>ercas Software Solutions GmbH</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Bilanzbuchhalter (m/w/d) Vollzeit in</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>kontakt@ercas.com</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Bewerbung als Bilanzbuchhalter (m/w/d) Vollzeit in - ercas Software Solutions GmbH</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Bilanzbuchhalter (m/w/d) Vollzeit in in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>ercas Software Solutions GmbH</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Architekt*in Wohnungsbau (m/w/d) Vollzeit in</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>kontakt@ercas.com</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Bewerbung als Architekt*in Wohnungsbau (m/w/d) Vollzeit in - ercas Software Solutions GmbH</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Architekt*in Wohnungsbau (m/w/d) Vollzeit in in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>ercas Software Solutions GmbH</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Baukalkulator (m/w/d) Vollzeit in</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>kontakt@ercas.com</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Bewerbung als Baukalkulator (m/w/d) Vollzeit in - ercas Software Solutions GmbH</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Baukalkulator (m/w/d) Vollzeit in in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>ercas Software Solutions GmbH</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Wirtschaftsingenieur (m/w/d) – Unit A / B / C Vollzeit in</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>kontakt@ercas.com</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Bewerbung als Wirtschaftsingenieur (m/w/d) – Unit A / B / C Vollzeit in - ercas Software Solutions GmbH</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Wirtschaftsingenieur (m/w/d) – Unit A / B / C Vollzeit in in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>ercas Software Solutions GmbH</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Wirtschaftsingenieur (m/w/d) – Unit A / B / C</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>kontakt@ercas.com</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Bewerbung als Wirtschaftsingenieur (m/w/d) – Unit A / B / C - ercas Software Solutions GmbH</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Wirtschaftsingenieur (m/w/d) – Unit A / B / C in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Schaeffler Technologies AG &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Duales Studium (DHBW) - Data Science und künstliche Intelligenz (m/w/d) 2026</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>info.de@schaeffler.com</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Bewerbung als Duales Studium (DHBW) - Data Science und künstliche Intelligenz (m/w/d) 2026 - Schaeffler Technologies AG &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Duales Studium (DHBW) - Data Science und künstliche Intelligenz (m/w/d) 2026 in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>M.IT Connect GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Ausbildung zum Kaufmann für IT-System-Management (m/w/d)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Bewerbung als Ausbildung zum Kaufmann für IT-System-Management (m/w/d) - M.IT Connect GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Ausbildung zum Kaufmann für IT-System-Management (m/w/d) in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>M.IT Connect GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>IT-Consultant (m/w/d) für Microsoft 365</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Bewerbung als IT-Consultant (m/w/d) für Microsoft 365 - M.IT Connect GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als IT-Consultant (m/w/d) für Microsoft 365 in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>M.IT Connect GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Ausbildung zum Fachinformatiker (m/w/d) für Systemintegration</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Bewerbung als Ausbildung zum Fachinformatiker (m/w/d) für Systemintegration - M.IT Connect GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Ausbildung zum Fachinformatiker (m/w/d) für Systemintegration in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>M.IT Connect GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Ausbildung zum Fachinformatiker (m/w/d) für Daten- und Prozessanalyse</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Bewerbung als Ausbildung zum Fachinformatiker (m/w/d) für Daten- und Prozessanalyse - M.IT Connect GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Ausbildung zum Fachinformatiker (m/w/d) für Daten- und Prozessanalyse in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>M.IT Connect GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Ausbildung zum Fachinformatiker (m/w/d) für Anwendungsentwicklung</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Bewerbung als Ausbildung zum Fachinformatiker (m/w/d) für Anwendungsentwicklung - M.IT Connect GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Ausbildung zum Fachinformatiker (m/w/d) für Anwendungsentwicklung in Vollzeit.
 Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
 Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
 In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
@@ -2523,7 +3604,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-15 16:44</t>
+          <t>2026-05-15 16:50</t>
         </is>
       </c>
     </row>
@@ -2534,7 +3615,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>19</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4">
@@ -2544,7 +3625,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
@@ -2554,7 +3635,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Job Scraper v5: 3 co | 41 jobs | 05-15 16:52
</commit_message>
<xml_diff>
--- a/download/Bewerbungen_Junior_IT.xlsx
+++ b/download/Bewerbungen_Junior_IT.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Statistiken" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bewerbungen'!$A$1:$N$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bewerbungen'!$A$1:$N$42</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N31"/>
+  <dimension ref="A1:N42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2534,9 +2534,718 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>AlphaConsult KG</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Technischer Support (m/w/d)</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Quelle: Arbeitsagentur</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>info@alphaconsult.org</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr"/>
+      <c r="G32" s="2" t="inlineStr"/>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>http://www.alphaconsult.org/</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Wilhelmstraße 4, 91413 Neustadt an der Aisch</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Technischer Support (m/w/d) in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr"/>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15 16:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>AlphaConsult KG</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Systemadministrator (m/w/d)</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Quelle: Arbeitsagentur</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>info@alphaconsult.org</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr"/>
+      <c r="F33" s="2" t="inlineStr"/>
+      <c r="G33" s="2" t="inlineStr"/>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>http://www.alphaconsult.org/</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>Wilhelmstraße 4, 91413 Neustadt an der Aisch</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Systemadministrator (m/w/d) in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr"/>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15 16:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Siemens AG</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Ressourcen für Entwickler</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Ressourcen für Entwickler</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>contact@siemens.com</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr"/>
+      <c r="G34" s="2" t="inlineStr"/>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.siemens.com/de-de/company/global-locations/germany/erlangen</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>Schuhstraße 60 Erlangen</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Ressourcen für Entwickler in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.siemens.com/de-de/support/documentation-downloads#toc-6ucoyS6q1lzPjocN4Llbyh-heading-3</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15 16:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Siemens AG</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Systems Engineering Digital Thread</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Systems Engineering Digital Thread</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>contact@siemens.com</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr"/>
+      <c r="F35" s="2" t="inlineStr"/>
+      <c r="G35" s="2" t="inlineStr"/>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.siemens.com/de-de/company/global-locations/germany/erlangen</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>Schuhstraße 60 Erlangen</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Systems Engineering Digital Thread in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.siemens.com/de-de/digital-thread/mbse/</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15 16:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Siemens AG</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Systems engineering software</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Systems engineering software</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>contact@siemens.com</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr"/>
+      <c r="G36" s="2" t="inlineStr"/>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.siemens.com/de-de/company/global-locations/germany/erlangen</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>Schuhstraße 60 Erlangen</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Systems engineering software in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.siemens.com/de-de/solutions/systems-engineering/</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15 16:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Siemens AG</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Service Engineering</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Service Engineering</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>contact@siemens.com</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr"/>
+      <c r="F37" s="2" t="inlineStr"/>
+      <c r="G37" s="2" t="inlineStr"/>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>https://www.siemens.com/de-de/company/global-locations/germany/erlangen</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>Schuhstraße 60 Erlangen</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Service Engineering in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>https://www.siemens.com/de-de/solutions/service-engineering/</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="N37" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15 16:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Siemens AG</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>allForschung und Entwicklung für die ZukunftSiemens-Forscherinnen und Forscher arbeiten eng mit Kunden und Partnern zusammen, um Technologie mit Sinn</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>allForschung und Entwicklung für die ZukunftSiemens-Forscherinnen und Forscher arbeiten eng mit Kunden und Partnern zusammen, um Technologie mit Sinn für Industrie, Infrastruktur, Transport und Gesundheitswesen zu entwickeln.</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>contact@siemens.com</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr"/>
+      <c r="G38" s="2" t="inlineStr"/>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>https://www.siemens.com/de-de/company/global-locations/germany/erlangen</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>Schuhstraße 60 Erlangen</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als allForschung und Entwicklung für die ZukunftSiemens-Forscherinnen und Forscher arbeiten eng mit Kunden und Partnern zusammen, um Technologie mit Sinn in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>https://www.siemens.com/en-us/company/innovation/research-development/</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15 16:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Siemens Healthineers AG</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Field Service Engineering &amp; Customer ServiceUnsere Field Service Engineering und Customer Service Teams spielen eine entscheidende Rolle dabei, Gesund</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Field Service Engineering &amp; Customer ServiceUnsere Field Service Engineering und Customer Service Teams spielen eine entscheidende Rolle dabei, Gesundheitseinrichtungen bei der Bereitstellung einer hochwertigen Versorgung zu unterstützen. Mit einem starken Kundenfokus bieten sie fachkundige Unterstützung, smarte Lösungen und ein hohes Maß an Engagement im Service.Mehr erfahren</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr"/>
+      <c r="E39" s="2" t="inlineStr"/>
+      <c r="F39" s="2" t="inlineStr"/>
+      <c r="G39" s="2" t="inlineStr"/>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>https://www.siemens-healthineers.com/deu</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>Hartmannstraße 16 Erlangen</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Field Service Engineering &amp; Customer ServiceUnsere Field Service Engineering und Customer Service Teams spielen eine entscheidende Rolle dabei, Gesund in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>https://www.siemens-healthineers.com/deu/careers/customer-services</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="N39" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15 16:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Siemens Healthineers AG</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Field Service Engineering &amp; Customer Service</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Field Service Engineering &amp; Customer Service</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr"/>
+      <c r="E40" s="2" t="inlineStr"/>
+      <c r="F40" s="2" t="inlineStr"/>
+      <c r="G40" s="2" t="inlineStr"/>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>https://www.siemens-healthineers.com/deu</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>Hartmannstraße 16 Erlangen</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Field Service Engineering &amp; Customer Service in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>https://www.siemens-healthineers.com/deu/careers/customer-services</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15 16:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Siemens Healthineers AG</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Software-Entwicklung, Cybersecurity und ITUnsere Tech-Teams gestalten die Zukunft des Gesundheitswesens. Unsere Software Engineers verwandeln komplexe</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Software-Entwicklung, Cybersecurity und ITUnsere Tech-Teams gestalten die Zukunft des Gesundheitswesens. Unsere Software Engineers verwandeln komplexe Ideen in reale Lösungen. Unsere Cybersecurity-Experten und -Expertinnen schützen unsere digitalen Systeme. Unsere IT-Fachkräfte bauen eine robuste Infrastruktur auf und sorgen so für einen reibungslosen Betrieb.Mehr erfahren</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr"/>
+      <c r="E41" s="2" t="inlineStr"/>
+      <c r="F41" s="2" t="inlineStr"/>
+      <c r="G41" s="2" t="inlineStr"/>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>https://www.siemens-healthineers.com/deu</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>Hartmannstraße 16 Erlangen</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Software-Entwicklung, Cybersecurity und ITUnsere Tech-Teams gestalten die Zukunft des Gesundheitswesens. Unsere Software Engineers verwandeln komplexe in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>https://www.siemens-healthineers.com/deu/careers/software-engineering-it-digital</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="N41" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15 16:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Siemens Healthineers AG</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Softwareentwickler*in (w/m/d) für System Software im Bereich Magnetresonanztomographie</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Quelle: Arbeitsagentur</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr"/>
+      <c r="E42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="inlineStr"/>
+      <c r="G42" s="2" t="inlineStr"/>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>https://www.siemens-healthineers.com/deu</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>Hartmannstraße 16 Erlangen</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Softwareentwickler*in (w/m/d) für System Software im Bereich Magnetresonanztomographie in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr"/>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15 16:52</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N31"/>
-  <conditionalFormatting sqref="H2:H31">
+  <autoFilter ref="A1:N42"/>
+  <conditionalFormatting sqref="H2:H42">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Zusage"</formula>
     </cfRule>
@@ -2553,13 +3262,13 @@
       <formula>"Interview absolviert"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M2:M31">
+  <conditionalFormatting sqref="M2:M42">
     <cfRule type="cellIs" priority="6" operator="equal" dxfId="0">
       <formula>"Ja"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2 H3 H4 H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2 H3 H4 H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 H40 H41 H42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Offen,Beworben,Interview eingeplant,Interview absolviert,Zusage,Absage,Kontaktiert,Wiedervorlage,Kein Interesse"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2573,7 +3282,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3561,6 +4270,364 @@
         <is>
           <t>Sehr geehrter Damen und Herren,
 ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Ausbildung zum Fachinformatiker (m/w/d) für Anwendungsentwicklung in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>AlphaConsult KG</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Technischer Support (m/w/d)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>info@alphaconsult.org</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Bewerbung als Technischer Support (m/w/d) - AlphaConsult KG</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Technischer Support (m/w/d) in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>AlphaConsult KG</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Systemadministrator (m/w/d)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>info@alphaconsult.org</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Bewerbung als Systemadministrator (m/w/d) - AlphaConsult KG</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Systemadministrator (m/w/d) in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Siemens AG</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Ressourcen für Entwickler</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>contact@siemens.com</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Bewerbung als Ressourcen für Entwickler - Siemens AG</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Ressourcen für Entwickler in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Siemens AG</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Systems Engineering Digital Thread</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>contact@siemens.com</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Bewerbung als Systems Engineering Digital Thread - Siemens AG</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Systems Engineering Digital Thread in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Siemens AG</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Systems engineering software</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>contact@siemens.com</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Bewerbung als Systems engineering software - Siemens AG</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Systems engineering software in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Siemens AG</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Service Engineering</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>contact@siemens.com</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Bewerbung als Service Engineering - Siemens AG</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Service Engineering in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Siemens AG</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>allForschung und Entwicklung für die ZukunftSiemens-Forscherinnen und Forscher arbeiten eng mit Kunden und Partnern zusammen, um Technologie mit Sinn</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>contact@siemens.com</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Bewerbung als allForschung und Entwicklung für die ZukunftSiemens-Forscherinnen und Forscher arbeiten eng mit Kunden und Partnern zusammen, um Technologie mit Sinn - Siemens AG</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als allForschung und Entwicklung für die ZukunftSiemens-Forscherinnen und Forscher arbeiten eng mit Kunden und Partnern zusammen, um Technologie mit Sinn in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Siemens Healthineers AG</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Field Service Engineering &amp; Customer ServiceUnsere Field Service Engineering und Customer Service Teams spielen eine entscheidende Rolle dabei, Gesund</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Bewerbung als Field Service Engineering &amp; Customer ServiceUnsere Field Service Engineering und Customer Service Teams spielen eine entscheidende Rolle dabei, Gesund - Siemens Healthineers AG</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Field Service Engineering &amp; Customer ServiceUnsere Field Service Engineering und Customer Service Teams spielen eine entscheidende Rolle dabei, Gesund in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Siemens Healthineers AG</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Field Service Engineering &amp; Customer Service</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Bewerbung als Field Service Engineering &amp; Customer Service - Siemens Healthineers AG</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Field Service Engineering &amp; Customer Service in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Siemens Healthineers AG</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Software-Entwicklung, Cybersecurity und ITUnsere Tech-Teams gestalten die Zukunft des Gesundheitswesens. Unsere Software Engineers verwandeln komplexe</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Bewerbung als Software-Entwicklung, Cybersecurity und ITUnsere Tech-Teams gestalten die Zukunft des Gesundheitswesens. Unsere Software Engineers verwandeln komplexe - Siemens Healthineers AG</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Software-Entwicklung, Cybersecurity und ITUnsere Tech-Teams gestalten die Zukunft des Gesundheitswesens. Unsere Software Engineers verwandeln komplexe in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Siemens Healthineers AG</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Softwareentwickler*in (w/m/d) für System Software im Bereich Magnetresonanztomographie</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Bewerbung als Softwareentwickler*in (w/m/d) für System Software im Bereich Magnetresonanztomographie - Siemens Healthineers AG</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Softwareentwickler*in (w/m/d) für System Software im Bereich Magnetresonanztomographie in Vollzeit.
 Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
 Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
 In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
@@ -3604,7 +4671,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-15 16:50</t>
+          <t>2026-05-15 16:52</t>
         </is>
       </c>
     </row>
@@ -3615,7 +4682,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>30</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4">
@@ -3635,7 +4702,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Job Scraper v5: 3 co | 47 jobs | 05-15 16:55
</commit_message>
<xml_diff>
--- a/download/Bewerbungen_Junior_IT.xlsx
+++ b/download/Bewerbungen_Junior_IT.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Statistiken" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bewerbungen'!$A$1:$N$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bewerbungen'!$A$1:$N$48</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N42"/>
+  <dimension ref="A1:N48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3243,9 +3243,395 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>SPS Germany GmbH</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>SAP Consultant PA | PY (gn)</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Quelle: Arbeitsagentur</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>datenschutz@sph-consulting.de</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr"/>
+      <c r="F43" s="2" t="inlineStr"/>
+      <c r="G43" s="2" t="inlineStr"/>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>https://www.spsglobal.com/de/transparenzinformation-sps-bamberg</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>Bamberg</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>Sehr geehrte Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als SAP Consultant PA | PY (gn) in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+      <c r="L43" s="2" t="inlineStr"/>
+      <c r="M43" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="N43" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15 16:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Robert Bosch GmbH</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Werkstudent IT Campus Management &amp; Digitalisierung (w/m/div.)Map PinStandort:Stuttgart-Feuerbach, Baden-WürttembergBriefcaseArbeitsbereich:Information</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Werkstudent IT Campus Management &amp; Digitalisierung (w/m/div.)Map PinStandort:Stuttgart-Feuerbach, Baden-WürttembergBriefcaseArbeitsbereich:InformationstechnologieCalendar AddJob veröffentlicht15.05.2026</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>kontakt@bosch.de</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr"/>
+      <c r="F44" s="2" t="inlineStr"/>
+      <c r="G44" s="2" t="inlineStr"/>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>http://www.bosch.de/</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>Gewerbegebiet Gewerbepark Brodswinden Süd, Robert-Bosch-Straße 1, 91522 Ansbach, Deutschland, 91522 Ansbach</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>Sehr geehrte Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Werkstudent IT Campus Management &amp; Digitalisierung (w/m/div.)Map PinStandort:Stuttgart-Feuerbach, Baden-WürttembergBriefcaseArbeitsbereich:Information in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>https://jobs.bosch.de/job/Werkstudent-IT-Campus-Management-Digitalisierung-w_m_div.-Stuttgart-Feuerbach?id=586683ae-90d0-4769-ab93-e406439ca3c8</t>
+        </is>
+      </c>
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="N44" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15 16:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Robert Bosch GmbH</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Pflichtpraktikum Agile Software Engineering und ManagementMap PinStandort:Abstatt bei Stuttgart, Baden-WürttembergBriefcaseArbeitsbereich:Informations</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Pflichtpraktikum Agile Software Engineering und ManagementMap PinStandort:Abstatt bei Stuttgart, Baden-WürttembergBriefcaseArbeitsbereich:InformationstechnologieCalendar AddJob veröffentlicht15.05.2026</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>kontakt@bosch.de</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr"/>
+      <c r="F45" s="2" t="inlineStr"/>
+      <c r="G45" s="2" t="inlineStr"/>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>http://www.bosch.de/</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>Gewerbegebiet Gewerbepark Brodswinden Süd, Robert-Bosch-Straße 1, 91522 Ansbach, Deutschland, 91522 Ansbach</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>Sehr geehrte Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Pflichtpraktikum Agile Software Engineering und ManagementMap PinStandort:Abstatt bei Stuttgart, Baden-WürttembergBriefcaseArbeitsbereich:Informations in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>https://jobs.bosch.de/job/Pflichtpraktikum-Agile-Software-Engineering-und-Management-Abstatt-bei-Stuttgart?id=161902dc-3dbf-49e0-a1f1-5fe116af4255</t>
+        </is>
+      </c>
+      <c r="M45" s="2" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="N45" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15 16:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Robert Bosch GmbH</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Werkstudent Machine Learning Engineering (w/m/div.) / REF283310J</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Quelle: Arbeitsagentur</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>kontakt@bosch.de</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr"/>
+      <c r="F46" s="2" t="inlineStr"/>
+      <c r="G46" s="2" t="inlineStr"/>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>http://www.bosch.de/</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>Gewerbegebiet Gewerbepark Brodswinden Süd, Robert-Bosch-Straße 1, 91522 Ansbach, Deutschland, 91522 Ansbach</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>Sehr geehrte Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Werkstudent Machine Learning Engineering (w/m/div.) / REF283310J in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr"/>
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="N46" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15 16:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Robert Bosch GmbH</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Werkstudent im Bereich SAP Process Navigator (w/m/div.) / REF278321Q</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Quelle: Arbeitsagentur</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>kontakt@bosch.de</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr"/>
+      <c r="F47" s="2" t="inlineStr"/>
+      <c r="G47" s="2" t="inlineStr"/>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>http://www.bosch.de/</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>Gewerbegebiet Gewerbepark Brodswinden Süd, Robert-Bosch-Straße 1, 91522 Ansbach, Deutschland, 91522 Ansbach</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>Sehr geehrte Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Werkstudent im Bereich SAP Process Navigator (w/m/div.) / REF278321Q in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+      <c r="L47" s="2" t="inlineStr"/>
+      <c r="M47" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="N47" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15 16:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Robert Bosch GmbH</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Ausbildung: Fachinformatiker 2027 (w/m/div.) Fachrichtung: Digitale Vernetzung / 2027_443</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Quelle: Arbeitsagentur</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>kontakt@bosch.de</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr"/>
+      <c r="F48" s="2" t="inlineStr"/>
+      <c r="G48" s="2" t="inlineStr"/>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>http://www.bosch.de/</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>Gewerbegebiet Gewerbepark Brodswinden Süd, Robert-Bosch-Straße 1, 91522 Ansbach, Deutschland, 91522 Ansbach</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>Sehr geehrte Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Ausbildung: Fachinformatiker 2027 (w/m/div.) Fachrichtung: Digitale Vernetzung / 2027_443 in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="inlineStr"/>
+      <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="N48" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-15 16:55</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N42"/>
-  <conditionalFormatting sqref="H2:H42">
+  <autoFilter ref="A1:N48"/>
+  <conditionalFormatting sqref="H2:H48">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Zusage"</formula>
     </cfRule>
@@ -3262,13 +3648,13 @@
       <formula>"Interview absolviert"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M2:M42">
+  <conditionalFormatting sqref="M2:M48">
     <cfRule type="cellIs" priority="6" operator="equal" dxfId="0">
       <formula>"Ja"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2 H3 H4 H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 H40 H41 H42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2 H3 H4 H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 H40 H41 H42 H43 H44 H45 H46 H47 H48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Offen,Beworben,Interview eingeplant,Interview absolviert,Zusage,Absage,Kontaktiert,Wiedervorlage,Kein Interesse"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3282,7 +3668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4628,6 +5014,210 @@
         <is>
           <t>Sehr geehrter Damen und Herren,
 ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Softwareentwickler*in (w/m/d) für System Software im Bereich Magnetresonanztomographie in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>SPS Germany GmbH</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>SAP Consultant PA | PY (gn)</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>datenschutz@sph-consulting.de</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Bewerbung als SAP Consultant PA | PY (gn) - SPS Germany GmbH</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Sehr geehrte Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als SAP Consultant PA | PY (gn) in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Robert Bosch GmbH</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Werkstudent IT Campus Management &amp; Digitalisierung (w/m/div.)Map PinStandort:Stuttgart-Feuerbach, Baden-WürttembergBriefcaseArbeitsbereich:Information</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>kontakt@bosch.de</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Bewerbung als Werkstudent IT Campus Management &amp; Digitalisierung (w/m/div.)Map PinStandort:Stuttgart-Feuerbach, Baden-WürttembergBriefcaseArbeitsbereich:Information - Robert Bosch GmbH</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Sehr geehrte Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Werkstudent IT Campus Management &amp; Digitalisierung (w/m/div.)Map PinStandort:Stuttgart-Feuerbach, Baden-WürttembergBriefcaseArbeitsbereich:Information in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Robert Bosch GmbH</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Pflichtpraktikum Agile Software Engineering und ManagementMap PinStandort:Abstatt bei Stuttgart, Baden-WürttembergBriefcaseArbeitsbereich:Informations</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>kontakt@bosch.de</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Bewerbung als Pflichtpraktikum Agile Software Engineering und ManagementMap PinStandort:Abstatt bei Stuttgart, Baden-WürttembergBriefcaseArbeitsbereich:Informations - Robert Bosch GmbH</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Sehr geehrte Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Pflichtpraktikum Agile Software Engineering und ManagementMap PinStandort:Abstatt bei Stuttgart, Baden-WürttembergBriefcaseArbeitsbereich:Informations in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Robert Bosch GmbH</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Werkstudent Machine Learning Engineering (w/m/div.) / REF283310J</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>kontakt@bosch.de</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Bewerbung als Werkstudent Machine Learning Engineering (w/m/div.) / REF283310J - Robert Bosch GmbH</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Sehr geehrte Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Werkstudent Machine Learning Engineering (w/m/div.) / REF283310J in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Robert Bosch GmbH</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Werkstudent im Bereich SAP Process Navigator (w/m/div.) / REF278321Q</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>kontakt@bosch.de</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Bewerbung als Werkstudent im Bereich SAP Process Navigator (w/m/div.) / REF278321Q - Robert Bosch GmbH</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Sehr geehrte Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Werkstudent im Bereich SAP Process Navigator (w/m/div.) / REF278321Q in Vollzeit.
+Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
+Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
+In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
+Ich arbeite selbstständig und kommuniziere offen. Das haben mir auch meine Betreuer in den Praxisphasen zurückgemeldet. Einen Führerschein der Klasse B besitze ich aktuell nicht, bin aber bereit, diesen zeitnah zu erwerben.
+Meine vollständigen Unterlagen finden Sie im Anhang. Ich freue mich auf ein persönliches Gespräch.
+Mit freundlichen Grüßen,</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Robert Bosch GmbH</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Ausbildung: Fachinformatiker 2027 (w/m/div.) Fachrichtung: Digitale Vernetzung / 2027_443</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>kontakt@bosch.de</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Bewerbung als Ausbildung: Fachinformatiker 2027 (w/m/div.) Fachrichtung: Digitale Vernetzung / 2027_443 - Robert Bosch GmbH</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Sehr geehrte Damen und Herren,
+ich sende Ihnen hiermit meine Bewerbungsunterlagen für die Stelle als Ausbildung: Fachinformatiker 2027 (w/m/div.) Fachrichtung: Digitale Vernetzung / 2027_443 in Vollzeit.
 Ich schließe meine Ausbildung zum Fachinformatiker für Systemintegration bald ab. Das Fachgespräch findet am 11. Juni 2026 statt, ab diesem Zeitpunkt stehe ich für eine Einstellung zur Verfügung.
 Während meiner Ausbildung hatte ich Berührungspunkte mit verschiedenen IT-Bereichen: Systemintegration, Webentwicklung und Datenbankentwicklung.
 In meiner letzten Praxisphase habe ich mich mit Azure beschäftigt, was direkt in mein IHK-Abschlussprojekt geflossen ist: die automatisierte Anwendungsbereitstellung via App Attach in Azure Virtual Desktop, von der Planung bis zur Dokumentation eigenständig umgesetzt.
@@ -4671,7 +5261,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-15 16:52</t>
+          <t>2026-05-15 16:55</t>
         </is>
       </c>
     </row>
@@ -4682,7 +5272,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>41</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4">
@@ -4692,7 +5282,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5">
@@ -4702,7 +5292,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6">

</xml_diff>